<commit_message>
useless texts taken out
</commit_message>
<xml_diff>
--- a/apps/admin/public/templates/igo-packages.xlsx
+++ b/apps/admin/public/templates/igo-packages.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="1" r:id="R9c78180e6eb34ca7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R2db7849056b442f1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages" sheetId="1" r:id="R9f5a66edb94b49c3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R0fa5f6938ca24d51"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="200" formatCode="@"/>
     <numFmt numFmtId="201" formatCode="0.00"/>
@@ -296,7 +296,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23" hidden="0" customWidth="1"/>
@@ -313,10 +313,10 @@
         <v>Parcel reference</v>
       </c>
       <c r="B1" s="4" t="str">
-        <v>Recipient name</v>
+        <v>Customer name</v>
       </c>
       <c r="C1" s="4" t="str">
-        <v>Recipient phone</v>
+        <v>Customer phone</v>
       </c>
       <c r="D1" s="4" t="str">
         <v>Destination</v>
@@ -4840,7 +4840,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25" hidden="0" customWidth="1"/>

</xml_diff>